<commit_message>
Switch to uv + ortools 9.15
- pyproject: ortools>=9.14, pandas>=2, numpy>=1.26 (drop the 9.10 downgrade pins).
- uv.lock committed; `uv sync --extra dev` builds .venv (ortools 9.15.6755,
  numpy 2.4.6, pandas 3.0.5). All 24 tests pass, results unchanged.
- ortools 9.15 loads fine in an isolated venv; the earlier WinError 127 was a
  conda-base DLL clash. README updated to the uv workflow.
- requirements.txt regenerated via `uv export` for pip users.
- .python-version pins 3.11.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/schedule_output.xlsx
+++ b/examples/schedule_output.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fleet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="schedules" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coverage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="fleet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="schedules" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="coverage" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,16 +23,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,21 +48,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -436,47 +424,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>tables_available</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>capacity</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>objective</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>total_shortage</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>total_surplus</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>realized_theo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>realized_hands</t>
         </is>
@@ -596,42 +584,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>table</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>pod</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>preferred_open_hours</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>theo_per_open_hour</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>patron_hands_per_hour</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>has_history</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>available_from</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>available_to</t>
         </is>
@@ -661,7 +649,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" s="2" t="n">
+      <c r="H2" s="1" t="n">
         <v>46266</v>
       </c>
     </row>
@@ -1152,7 +1140,7 @@
       <c r="F21" t="b">
         <v>0</v>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G21" s="1" t="n">
         <v>46267</v>
       </c>
       <c r="H21" t="inlineStr"/>
@@ -1172,47 +1160,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>table</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>pod</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>score</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>has_history</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>preferred_open_hours</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>shift</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>shift_open_hours</t>
         </is>
@@ -3342,42 +3330,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>day</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>hour_index</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>clock</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>demand</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>capacity</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>tables_open</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>shortage</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>surplus</t>
         </is>

</xml_diff>